<commit_message>
Refactor: clear all metadata, student lists, grades, and attendance from Excel templates
</commit_message>
<xml_diff>
--- a/Registro Primaria.xlsx
+++ b/Registro Primaria.xlsx
@@ -2517,7 +2517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A7:AD25"/>
+  <dimension ref="A7:BQ54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="2.6640625" customWidth="1" style="147" min="1" max="39"/>
@@ -2554,27 +2554,48 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
     <row r="23" ht="17.4" customHeight="1" s="147">
-      <c r="Q23" s="172" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Maestro  Elmer Tugri </t>
-        </is>
-      </c>
+      <c r="Q23" s="172" t="n"/>
     </row>
     <row r="24" ht="17.4" customHeight="1" s="147">
-      <c r="Q24" s="172" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Maestro de Grado</t>
-        </is>
-      </c>
+      <c r="Q24" s="172" t="n"/>
     </row>
     <row r="25" ht="17.4" customHeight="1" s="147">
-      <c r="Q25" s="172" t="inlineStr">
-        <is>
-          <t>Grupo: 1°</t>
-        </is>
-      </c>
-    </row>
+      <c r="Q25" s="172" t="n"/>
+    </row>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="L7:T7"/>
@@ -2599,7 +2620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B3:Q56"/>
+  <dimension ref="B3:BQ56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="0.44140625" customWidth="1" style="147" min="1" max="1"/>
@@ -2881,46 +2902,14 @@
       <c r="G15" s="154" t="n"/>
       <c r="H15" s="154" t="n"/>
       <c r="I15" s="162" t="n"/>
-      <c r="J15" s="14" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K15" s="14" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="L15" s="14" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="M15" s="14" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="N15" s="14" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="O15" s="14" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="P15" s="14" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="Q15" s="14" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
+      <c r="J15" s="14" t="n"/>
+      <c r="K15" s="14" t="n"/>
+      <c r="L15" s="14" t="n"/>
+      <c r="M15" s="14" t="n"/>
+      <c r="N15" s="14" t="n"/>
+      <c r="O15" s="14" t="n"/>
+      <c r="P15" s="14" t="n"/>
+      <c r="Q15" s="14" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="9" t="n">
@@ -5466,7 +5455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R137"/>
+  <dimension ref="A1:BQ137"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="28.77734375" customWidth="1" style="147" min="1" max="1"/>
@@ -9063,7 +9052,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P152"/>
+  <dimension ref="A1:BQ152"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="147" min="1" max="1"/>
@@ -9349,6 +9338,7 @@
       <c r="F17" s="192" t="n"/>
       <c r="G17" s="192" t="n"/>
     </row>
+    <row r="18"/>
     <row r="19" ht="19.95" customHeight="1" s="147">
       <c r="A19" s="253" t="inlineStr">
         <is>
@@ -9392,16 +9382,8 @@
           <t>INGLÉS</t>
         </is>
       </c>
-      <c r="E20" s="125" t="inlineStr">
-        <is>
-          <t>TECNOLOGÍA</t>
-        </is>
-      </c>
-      <c r="F20" s="125" t="inlineStr">
-        <is>
-          <t>OBSERVACIONES</t>
-        </is>
-      </c>
+      <c r="E20" s="125" t="n"/>
+      <c r="F20" s="125" t="n"/>
     </row>
     <row r="21" ht="13.95" customHeight="1" s="147">
       <c r="A21" s="192">
@@ -12257,7 +12239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L134"/>
+  <dimension ref="A1:BQ134"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" style="147" min="1" max="1"/>
@@ -13235,6 +13217,7 @@
       <c r="D46" s="130" t="n"/>
       <c r="E46" s="130" t="n"/>
     </row>
+    <row r="47"/>
     <row r="48" ht="19.95" customHeight="1" s="147">
       <c r="A48" s="258" t="n"/>
       <c r="B48" s="193" t="n"/>
@@ -13872,7 +13855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:BQ54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="22" customWidth="1" style="147" min="1" max="1"/>
@@ -14314,6 +14297,31 @@
       <c r="M29" s="193" t="n"/>
       <c r="N29" s="194" t="n"/>
     </row>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
   </sheetData>
   <mergeCells count="19">
     <mergeCell ref="A24:N24"/>
@@ -14347,13 +14355,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:AZ43"/>
+  <dimension ref="A1:AZ43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="6.44140625" customWidth="1" style="147" min="1" max="1"/>
     <col width="1.6640625" customWidth="1" style="147" min="2" max="63"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
     <row r="4" ht="18" customHeight="1" s="147">
       <c r="A4" s="175" t="inlineStr">
         <is>
@@ -14432,6 +14443,7 @@
       <c r="AX8" s="173" t="n"/>
       <c r="AY8" s="173" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="19.5" customHeight="1" s="147">
       <c r="A10" t="inlineStr">
         <is>
@@ -15336,7 +15348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:X33"/>
+  <dimension ref="A1:X33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="1.6640625" customWidth="1" style="147" min="1" max="14"/>
@@ -15897,7 +15909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:BQ124"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="44.6640625" customWidth="1" style="147" min="1" max="1"/>
@@ -16502,7 +16514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:H28"/>
+  <dimension ref="A4:BQ54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="4" ht="18" customHeight="1" s="147">
@@ -16712,6 +16724,30 @@
     </row>
     <row r="29" ht="25.05" customHeight="1" s="147"/>
     <row r="30" ht="25.05" customHeight="1" s="147"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A4:H4"/>
@@ -16728,7 +16764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="147" min="1" max="1"/>
@@ -16794,180 +16830,100 @@
       <c r="A5" s="84" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="192" t="inlineStr">
-        <is>
-          <t>BEJERANO, Jose</t>
-        </is>
-      </c>
+      <c r="B5" s="192" t="n"/>
       <c r="C5" s="193" t="n"/>
       <c r="D5" s="194" t="n"/>
-      <c r="E5" s="197" t="inlineStr">
-        <is>
-          <t>1-234-567</t>
-        </is>
-      </c>
+      <c r="E5" s="197" t="n"/>
       <c r="F5" s="193" t="n"/>
     </row>
     <row r="6" ht="16.05" customHeight="1" s="147">
       <c r="A6" s="86" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="196" t="inlineStr">
-        <is>
-          <t>GONZALEZ, Maria</t>
-        </is>
-      </c>
+      <c r="B6" s="196" t="n"/>
       <c r="C6" s="193" t="n"/>
       <c r="D6" s="194" t="n"/>
-      <c r="E6" s="195" t="inlineStr">
-        <is>
-          <t>4-789-012</t>
-        </is>
-      </c>
+      <c r="E6" s="195" t="n"/>
       <c r="F6" s="193" t="n"/>
     </row>
     <row r="7" ht="16.05" customHeight="1" s="147">
       <c r="A7" s="84" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="192" t="inlineStr">
-        <is>
-          <t>PINTO, Luis</t>
-        </is>
-      </c>
+      <c r="B7" s="192" t="n"/>
       <c r="C7" s="193" t="n"/>
       <c r="D7" s="194" t="n"/>
-      <c r="E7" s="197" t="inlineStr">
-        <is>
-          <t>9-345-678</t>
-        </is>
-      </c>
+      <c r="E7" s="197" t="n"/>
       <c r="F7" s="193" t="n"/>
     </row>
     <row r="8" ht="16.05" customHeight="1" s="147">
       <c r="A8" s="86" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="196" t="inlineStr">
-        <is>
-          <t>SANTOS, Ana</t>
-        </is>
-      </c>
+      <c r="B8" s="196" t="n"/>
       <c r="C8" s="193" t="n"/>
       <c r="D8" s="194" t="n"/>
-      <c r="E8" s="195" t="inlineStr">
-        <is>
-          <t>8-901-234</t>
-        </is>
-      </c>
+      <c r="E8" s="195" t="n"/>
       <c r="F8" s="193" t="n"/>
     </row>
     <row r="9" ht="16.05" customHeight="1" s="147">
       <c r="A9" s="84" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="192" t="inlineStr">
-        <is>
-          <t>TUGRI, Carlos</t>
-        </is>
-      </c>
+      <c r="B9" s="192" t="n"/>
       <c r="C9" s="193" t="n"/>
       <c r="D9" s="194" t="n"/>
-      <c r="E9" s="197" t="inlineStr">
-        <is>
-          <t>12-345-678</t>
-        </is>
-      </c>
+      <c r="E9" s="197" t="n"/>
       <c r="F9" s="193" t="n"/>
     </row>
     <row r="10" ht="16.05" customHeight="1" s="147">
       <c r="A10" s="86" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="196" t="inlineStr">
-        <is>
-          <t>ZURDO, Rosa</t>
-        </is>
-      </c>
+      <c r="B10" s="196" t="n"/>
       <c r="C10" s="193" t="n"/>
       <c r="D10" s="194" t="n"/>
-      <c r="E10" s="195" t="inlineStr">
-        <is>
-          <t>4-111-222</t>
-        </is>
-      </c>
+      <c r="E10" s="195" t="n"/>
       <c r="F10" s="193" t="n"/>
     </row>
     <row r="11" ht="16.05" customHeight="1" s="147">
       <c r="A11" s="84" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="192" t="inlineStr">
-        <is>
-          <t>JIMENEZ, Juan</t>
-        </is>
-      </c>
+      <c r="B11" s="192" t="n"/>
       <c r="C11" s="193" t="n"/>
       <c r="D11" s="194" t="n"/>
-      <c r="E11" s="197" t="inlineStr">
-        <is>
-          <t>8-444-555</t>
-        </is>
-      </c>
+      <c r="E11" s="197" t="n"/>
       <c r="F11" s="193" t="n"/>
     </row>
     <row r="12" ht="16.05" customHeight="1" s="147">
       <c r="A12" s="86" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="196" t="inlineStr">
-        <is>
-          <t>MONTERO, Sofia</t>
-        </is>
-      </c>
+      <c r="B12" s="196" t="n"/>
       <c r="C12" s="193" t="n"/>
       <c r="D12" s="194" t="n"/>
-      <c r="E12" s="195" t="inlineStr">
-        <is>
-          <t>9-888-999</t>
-        </is>
-      </c>
+      <c r="E12" s="195" t="n"/>
       <c r="F12" s="193" t="n"/>
     </row>
     <row r="13" ht="16.05" customHeight="1" s="147">
       <c r="A13" s="84" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="192" t="inlineStr">
-        <is>
-          <t>SALDANA, Pedro</t>
-        </is>
-      </c>
+      <c r="B13" s="192" t="n"/>
       <c r="C13" s="193" t="n"/>
       <c r="D13" s="194" t="n"/>
-      <c r="E13" s="197" t="inlineStr">
-        <is>
-          <t>2-222-333</t>
-        </is>
-      </c>
+      <c r="E13" s="197" t="n"/>
       <c r="F13" s="193" t="n"/>
     </row>
     <row r="14" ht="16.05" customHeight="1" s="147">
       <c r="A14" s="86" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="196" t="inlineStr">
-        <is>
-          <t>SANTOS, Lucas</t>
-        </is>
-      </c>
+      <c r="B14" s="196" t="n"/>
       <c r="C14" s="193" t="n"/>
       <c r="D14" s="194" t="n"/>
-      <c r="E14" s="195" t="inlineStr">
-        <is>
-          <t>8-777-888</t>
-        </is>
-      </c>
+      <c r="E14" s="195" t="n"/>
       <c r="F14" s="193" t="n"/>
     </row>
     <row r="15" ht="16.05" customHeight="1" s="147">
@@ -17210,6 +17166,7 @@
       <c r="E38" s="195" t="n"/>
       <c r="F38" s="193" t="n"/>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="203" t="inlineStr">
         <is>
@@ -17217,6 +17174,20 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
   </sheetData>
   <mergeCells count="74">
     <mergeCell ref="B11:D11"/>
@@ -17305,7 +17276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y121"/>
+  <dimension ref="A1:BQ121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" style="147" min="1" max="1"/>
@@ -18531,9 +18502,7 @@
         <v/>
       </c>
       <c r="L15" s="196" t="n"/>
-      <c r="N15" s="86" t="n">
-        <v>11</v>
-      </c>
+      <c r="N15" s="86" t="n"/>
       <c r="O15" s="87">
         <f>IF('MAESTRO 1°'!B15="","",'MAESTRO 1°'!B15)</f>
         <v/>
@@ -18621,9 +18590,7 @@
         <v/>
       </c>
       <c r="L16" s="192" t="n"/>
-      <c r="N16" s="84" t="n">
-        <v>12</v>
-      </c>
+      <c r="N16" s="84" t="n"/>
       <c r="O16" s="85">
         <f>IF('MAESTRO 1°'!B16="","",'MAESTRO 1°'!B16)</f>
         <v/>
@@ -18711,9 +18678,7 @@
         <v/>
       </c>
       <c r="L17" s="196" t="n"/>
-      <c r="N17" s="86" t="n">
-        <v>13</v>
-      </c>
+      <c r="N17" s="86" t="n"/>
       <c r="O17" s="87">
         <f>IF('MAESTRO 1°'!B17="","",'MAESTRO 1°'!B17)</f>
         <v/>
@@ -18801,9 +18766,7 @@
         <v/>
       </c>
       <c r="L18" s="192" t="n"/>
-      <c r="N18" s="84" t="n">
-        <v>14</v>
-      </c>
+      <c r="N18" s="84" t="n"/>
       <c r="O18" s="85">
         <f>IF('MAESTRO 1°'!B18="","",'MAESTRO 1°'!B18)</f>
         <v/>
@@ -18891,9 +18854,7 @@
         <v/>
       </c>
       <c r="L19" s="196" t="n"/>
-      <c r="N19" s="86" t="n">
-        <v>15</v>
-      </c>
+      <c r="N19" s="86" t="n"/>
       <c r="O19" s="87">
         <f>IF('MAESTRO 1°'!B19="","",'MAESTRO 1°'!B19)</f>
         <v/>
@@ -18981,9 +18942,7 @@
         <v/>
       </c>
       <c r="L20" s="192" t="n"/>
-      <c r="N20" s="84" t="n">
-        <v>16</v>
-      </c>
+      <c r="N20" s="84" t="n"/>
       <c r="O20" s="85">
         <f>IF('MAESTRO 1°'!B20="","",'MAESTRO 1°'!B20)</f>
         <v/>
@@ -19071,9 +19030,7 @@
         <v/>
       </c>
       <c r="L21" s="196" t="n"/>
-      <c r="N21" s="86" t="n">
-        <v>17</v>
-      </c>
+      <c r="N21" s="86" t="n"/>
       <c r="O21" s="87">
         <f>IF('MAESTRO 1°'!B21="","",'MAESTRO 1°'!B21)</f>
         <v/>
@@ -19161,9 +19118,7 @@
         <v/>
       </c>
       <c r="L22" s="192" t="n"/>
-      <c r="N22" s="84" t="n">
-        <v>18</v>
-      </c>
+      <c r="N22" s="84" t="n"/>
       <c r="O22" s="85">
         <f>IF('MAESTRO 1°'!B22="","",'MAESTRO 1°'!B22)</f>
         <v/>
@@ -19251,9 +19206,7 @@
         <v/>
       </c>
       <c r="L23" s="196" t="n"/>
-      <c r="N23" s="86" t="n">
-        <v>19</v>
-      </c>
+      <c r="N23" s="86" t="n"/>
       <c r="O23" s="87">
         <f>IF('MAESTRO 1°'!B23="","",'MAESTRO 1°'!B23)</f>
         <v/>
@@ -19341,9 +19294,7 @@
         <v/>
       </c>
       <c r="L24" s="192" t="n"/>
-      <c r="N24" s="84" t="n">
-        <v>20</v>
-      </c>
+      <c r="N24" s="84" t="n"/>
       <c r="O24" s="85">
         <f>IF('MAESTRO 1°'!B24="","",'MAESTRO 1°'!B24)</f>
         <v/>
@@ -19431,9 +19382,7 @@
         <v/>
       </c>
       <c r="L25" s="196" t="n"/>
-      <c r="N25" s="86" t="n">
-        <v>21</v>
-      </c>
+      <c r="N25" s="86" t="n"/>
       <c r="O25" s="87">
         <f>IF('MAESTRO 1°'!B25="","",'MAESTRO 1°'!B25)</f>
         <v/>
@@ -19521,9 +19470,7 @@
         <v/>
       </c>
       <c r="L26" s="192" t="n"/>
-      <c r="N26" s="84" t="n">
-        <v>22</v>
-      </c>
+      <c r="N26" s="84" t="n"/>
       <c r="O26" s="85">
         <f>IF('MAESTRO 1°'!B26="","",'MAESTRO 1°'!B26)</f>
         <v/>
@@ -19611,9 +19558,7 @@
         <v/>
       </c>
       <c r="L27" s="196" t="n"/>
-      <c r="N27" s="86" t="n">
-        <v>23</v>
-      </c>
+      <c r="N27" s="86" t="n"/>
       <c r="O27" s="87">
         <f>IF('MAESTRO 1°'!B27="","",'MAESTRO 1°'!B27)</f>
         <v/>
@@ -19701,9 +19646,7 @@
         <v/>
       </c>
       <c r="L28" s="192" t="n"/>
-      <c r="N28" s="84" t="n">
-        <v>24</v>
-      </c>
+      <c r="N28" s="84" t="n"/>
       <c r="O28" s="85">
         <f>IF('MAESTRO 1°'!B28="","",'MAESTRO 1°'!B28)</f>
         <v/>
@@ -19791,9 +19734,7 @@
         <v/>
       </c>
       <c r="L29" s="196" t="n"/>
-      <c r="N29" s="86" t="n">
-        <v>25</v>
-      </c>
+      <c r="N29" s="86" t="n"/>
       <c r="O29" s="87">
         <f>IF('MAESTRO 1°'!B29="","",'MAESTRO 1°'!B29)</f>
         <v/>
@@ -19881,9 +19822,7 @@
         <v/>
       </c>
       <c r="L30" s="192" t="n"/>
-      <c r="N30" s="84" t="n">
-        <v>26</v>
-      </c>
+      <c r="N30" s="84" t="n"/>
       <c r="O30" s="85">
         <f>IF('MAESTRO 1°'!B30="","",'MAESTRO 1°'!B30)</f>
         <v/>
@@ -19971,9 +19910,7 @@
         <v/>
       </c>
       <c r="L31" s="196" t="n"/>
-      <c r="N31" s="86" t="n">
-        <v>27</v>
-      </c>
+      <c r="N31" s="86" t="n"/>
       <c r="O31" s="87">
         <f>IF('MAESTRO 1°'!B31="","",'MAESTRO 1°'!B31)</f>
         <v/>
@@ -20061,9 +19998,7 @@
         <v/>
       </c>
       <c r="L32" s="192" t="n"/>
-      <c r="N32" s="84" t="n">
-        <v>28</v>
-      </c>
+      <c r="N32" s="84" t="n"/>
       <c r="O32" s="85">
         <f>IF('MAESTRO 1°'!B32="","",'MAESTRO 1°'!B32)</f>
         <v/>
@@ -20151,9 +20086,7 @@
         <v/>
       </c>
       <c r="L33" s="196" t="n"/>
-      <c r="N33" s="86" t="n">
-        <v>29</v>
-      </c>
+      <c r="N33" s="86" t="n"/>
       <c r="O33" s="87">
         <f>IF('MAESTRO 1°'!B33="","",'MAESTRO 1°'!B33)</f>
         <v/>
@@ -20241,9 +20174,7 @@
         <v/>
       </c>
       <c r="L34" s="192" t="n"/>
-      <c r="N34" s="84" t="n">
-        <v>30</v>
-      </c>
+      <c r="N34" s="84" t="n"/>
       <c r="O34" s="85">
         <f>IF('MAESTRO 1°'!B34="","",'MAESTRO 1°'!B34)</f>
         <v/>
@@ -20331,9 +20262,7 @@
         <v/>
       </c>
       <c r="L35" s="196" t="n"/>
-      <c r="N35" s="86" t="n">
-        <v>31</v>
-      </c>
+      <c r="N35" s="86" t="n"/>
       <c r="O35" s="87">
         <f>IF('MAESTRO 1°'!B35="","",'MAESTRO 1°'!B35)</f>
         <v/>
@@ -20421,9 +20350,7 @@
         <v/>
       </c>
       <c r="L36" s="192" t="n"/>
-      <c r="N36" s="84" t="n">
-        <v>32</v>
-      </c>
+      <c r="N36" s="84" t="n"/>
       <c r="O36" s="85">
         <f>IF('MAESTRO 1°'!B36="","",'MAESTRO 1°'!B36)</f>
         <v/>
@@ -20511,9 +20438,7 @@
         <v/>
       </c>
       <c r="L37" s="196" t="n"/>
-      <c r="N37" s="86" t="n">
-        <v>33</v>
-      </c>
+      <c r="N37" s="86" t="n"/>
       <c r="O37" s="87">
         <f>IF('MAESTRO 1°'!B37="","",'MAESTRO 1°'!B37)</f>
         <v/>
@@ -20601,9 +20526,7 @@
         <v/>
       </c>
       <c r="L38" s="192" t="n"/>
-      <c r="N38" s="84" t="n">
-        <v>34</v>
-      </c>
+      <c r="N38" s="84" t="n"/>
       <c r="O38" s="85">
         <f>IF('MAESTRO 1°'!B38="","",'MAESTRO 1°'!B38)</f>
         <v/>
@@ -20687,11 +20610,7 @@
       </c>
       <c r="K39" s="90" t="n"/>
       <c r="L39" s="90" t="n"/>
-      <c r="N39" s="209" t="inlineStr">
-        <is>
-          <t>PROMEDIO DEL GRUPO</t>
-        </is>
-      </c>
+      <c r="N39" s="209" t="n"/>
       <c r="O39" s="194" t="n"/>
       <c r="P39" s="90">
         <f>IFERROR(ROUND(AVERAGEIF(P5:P38,"&lt;&gt;"&amp;""),1),"")</f>
@@ -20768,46 +20687,14 @@
           <t>ESPAÑOL</t>
         </is>
       </c>
-      <c r="E42" s="95" t="inlineStr">
-        <is>
-          <t>Matemática</t>
-        </is>
-      </c>
-      <c r="F42" s="95" t="inlineStr">
-        <is>
-          <t>C.SOCIALES</t>
-        </is>
-      </c>
-      <c r="G42" s="95" t="inlineStr">
-        <is>
-          <t>C.NATURALES</t>
-        </is>
-      </c>
-      <c r="H42" s="95" t="inlineStr">
-        <is>
-          <t>Religión</t>
-        </is>
-      </c>
-      <c r="I42" s="95" t="inlineStr">
-        <is>
-          <t>Artística</t>
-        </is>
-      </c>
-      <c r="J42" s="95" t="inlineStr">
-        <is>
-          <t>TECNOLOGIA</t>
-        </is>
-      </c>
-      <c r="K42" s="95" t="inlineStr">
-        <is>
-          <t>E. FISICA</t>
-        </is>
-      </c>
-      <c r="L42" s="208" t="inlineStr">
-        <is>
-          <t>ESTADO</t>
-        </is>
-      </c>
+      <c r="E42" s="95" t="n"/>
+      <c r="F42" s="95" t="n"/>
+      <c r="G42" s="95" t="n"/>
+      <c r="H42" s="95" t="n"/>
+      <c r="I42" s="95" t="n"/>
+      <c r="J42" s="95" t="n"/>
+      <c r="K42" s="95" t="n"/>
+      <c r="L42" s="208" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="207" t="n"/>
@@ -20822,41 +20709,13 @@
           <t>FINAL</t>
         </is>
       </c>
-      <c r="E43" s="202" t="inlineStr">
-        <is>
-          <t>FINAL</t>
-        </is>
-      </c>
-      <c r="F43" s="202" t="inlineStr">
-        <is>
-          <t>FINAL</t>
-        </is>
-      </c>
-      <c r="G43" s="202" t="inlineStr">
-        <is>
-          <t>FINAL</t>
-        </is>
-      </c>
-      <c r="H43" s="202" t="inlineStr">
-        <is>
-          <t>FINAL</t>
-        </is>
-      </c>
-      <c r="I43" s="202" t="inlineStr">
-        <is>
-          <t>FINAL</t>
-        </is>
-      </c>
-      <c r="J43" s="202" t="inlineStr">
-        <is>
-          <t>FINAL</t>
-        </is>
-      </c>
-      <c r="K43" s="202" t="inlineStr">
-        <is>
-          <t>FINAL</t>
-        </is>
-      </c>
+      <c r="E43" s="202" t="n"/>
+      <c r="F43" s="202" t="n"/>
+      <c r="G43" s="202" t="n"/>
+      <c r="H43" s="202" t="n"/>
+      <c r="I43" s="202" t="n"/>
+      <c r="J43" s="202" t="n"/>
+      <c r="K43" s="202" t="n"/>
       <c r="L43" s="207" t="n"/>
     </row>
     <row r="44">
@@ -24384,7 +24243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL138"/>
+  <dimension ref="A1:BQ138"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="3.44140625" customWidth="1" style="147" min="1" max="1"/>
@@ -25580,9 +25439,7 @@
         <v/>
       </c>
       <c r="BK15" s="220" t="n"/>
-      <c r="BL15" s="3" t="n">
-        <v>13</v>
-      </c>
+      <c r="BL15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -25658,9 +25515,7 @@
         <v/>
       </c>
       <c r="BK16" s="220" t="n"/>
-      <c r="BL16" s="3" t="n">
-        <v>14</v>
-      </c>
+      <c r="BL16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -25736,9 +25591,7 @@
         <v/>
       </c>
       <c r="BK17" s="220" t="n"/>
-      <c r="BL17" s="3" t="n">
-        <v>15</v>
-      </c>
+      <c r="BL17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -25814,9 +25667,7 @@
         <v/>
       </c>
       <c r="BK18" s="220" t="n"/>
-      <c r="BL18" s="3" t="n">
-        <v>16</v>
-      </c>
+      <c r="BL18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -25893,9 +25744,7 @@
         <v/>
       </c>
       <c r="BK19" s="220" t="n"/>
-      <c r="BL19" s="3" t="n">
-        <v>17</v>
-      </c>
+      <c r="BL19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -25972,9 +25821,7 @@
         <v/>
       </c>
       <c r="BK20" s="220" t="n"/>
-      <c r="BL20" s="3" t="n">
-        <v>18</v>
-      </c>
+      <c r="BL20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -26051,9 +25898,7 @@
         <v/>
       </c>
       <c r="BK21" s="220" t="n"/>
-      <c r="BL21" s="3" t="n">
-        <v>19</v>
-      </c>
+      <c r="BL21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -26130,9 +25975,7 @@
         <v/>
       </c>
       <c r="BK22" s="220" t="n"/>
-      <c r="BL22" s="3" t="n">
-        <v>20</v>
-      </c>
+      <c r="BL22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -26209,9 +26052,7 @@
         <v/>
       </c>
       <c r="BK23" s="220" t="n"/>
-      <c r="BL23" s="3" t="n">
-        <v>21</v>
-      </c>
+      <c r="BL23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -26288,9 +26129,7 @@
         <v/>
       </c>
       <c r="BK24" s="220" t="n"/>
-      <c r="BL24" s="3" t="n">
-        <v>22</v>
-      </c>
+      <c r="BL24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -26367,9 +26206,7 @@
         <v/>
       </c>
       <c r="BK25" s="220" t="n"/>
-      <c r="BL25" s="3" t="n">
-        <v>23</v>
-      </c>
+      <c r="BL25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -26446,9 +26283,7 @@
         <v/>
       </c>
       <c r="BK26" s="220" t="n"/>
-      <c r="BL26" s="3" t="n">
-        <v>24</v>
-      </c>
+      <c r="BL26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -26525,9 +26360,7 @@
         <v/>
       </c>
       <c r="BK27" s="220" t="n"/>
-      <c r="BL27" s="3" t="n">
-        <v>25</v>
-      </c>
+      <c r="BL27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -26604,9 +26437,7 @@
         <v/>
       </c>
       <c r="BK28" s="220" t="n"/>
-      <c r="BL28" s="3" t="n">
-        <v>26</v>
-      </c>
+      <c r="BL28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -26683,9 +26514,7 @@
         <v/>
       </c>
       <c r="BK29" s="220" t="n"/>
-      <c r="BL29" s="3" t="n">
-        <v>27</v>
-      </c>
+      <c r="BL29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -26762,9 +26591,7 @@
         <v/>
       </c>
       <c r="BK30" s="220" t="n"/>
-      <c r="BL30" s="3" t="n">
-        <v>28</v>
-      </c>
+      <c r="BL30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -26841,9 +26668,7 @@
         <v/>
       </c>
       <c r="BK31" s="220" t="n"/>
-      <c r="BL31" s="3" t="n">
-        <v>29</v>
-      </c>
+      <c r="BL31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -26920,9 +26745,7 @@
         <v/>
       </c>
       <c r="BK32" s="220" t="n"/>
-      <c r="BL32" s="3" t="n">
-        <v>30</v>
-      </c>
+      <c r="BL32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -26999,9 +26822,7 @@
         <v/>
       </c>
       <c r="BK33" s="220" t="n"/>
-      <c r="BL33" s="3" t="n">
-        <v>31</v>
-      </c>
+      <c r="BL33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -27078,9 +26899,7 @@
         <v/>
       </c>
       <c r="BK34" s="220" t="n"/>
-      <c r="BL34" s="3" t="n">
-        <v>32</v>
-      </c>
+      <c r="BL34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -27157,9 +26976,7 @@
         <v/>
       </c>
       <c r="BK35" s="220" t="n"/>
-      <c r="BL35" s="3" t="n">
-        <v>33</v>
-      </c>
+      <c r="BL35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -27236,9 +27053,7 @@
         <v/>
       </c>
       <c r="BK36" s="220" t="n"/>
-      <c r="BL36" s="3" t="n">
-        <v>34</v>
-      </c>
+      <c r="BL36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -27315,9 +27130,7 @@
         <v/>
       </c>
       <c r="BK37" s="220" t="n"/>
-      <c r="BL37" s="3" t="n">
-        <v>35</v>
-      </c>
+      <c r="BL37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -27394,9 +27207,7 @@
         <v/>
       </c>
       <c r="BK38" s="220" t="n"/>
-      <c r="BL38" s="3" t="n">
-        <v>36</v>
-      </c>
+      <c r="BL38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -27473,9 +27284,7 @@
         <v/>
       </c>
       <c r="BK39" s="220" t="n"/>
-      <c r="BL39" s="3" t="n">
-        <v>37</v>
-      </c>
+      <c r="BL39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -27552,9 +27361,7 @@
         <v/>
       </c>
       <c r="BK40" s="220" t="n"/>
-      <c r="BL40" s="3" t="n">
-        <v>38</v>
-      </c>
+      <c r="BL40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -27631,9 +27438,7 @@
         <v/>
       </c>
       <c r="BK41" s="220" t="n"/>
-      <c r="BL41" s="3" t="n">
-        <v>39</v>
-      </c>
+      <c r="BL41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
@@ -27710,9 +27515,7 @@
         <v/>
       </c>
       <c r="BK42" s="220" t="n"/>
-      <c r="BL42" s="3" t="n">
-        <v>40</v>
-      </c>
+      <c r="BL42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
@@ -27786,9 +27589,7 @@
         <v/>
       </c>
       <c r="BK43" s="220" t="n"/>
-      <c r="BL43" s="220" t="n">
-        <v>41</v>
-      </c>
+      <c r="BL43" s="220" t="n"/>
     </row>
     <row r="44" ht="31.2" customHeight="1" s="147">
       <c r="A44" s="211" t="n"/>
@@ -27859,17 +27660,9 @@
       <c r="BF44" s="157" t="n"/>
       <c r="BG44" s="157" t="n"/>
       <c r="BH44" s="145" t="n"/>
-      <c r="BI44" s="214" t="inlineStr">
-        <is>
-          <t>SEGUNDO TRIMESTRE</t>
-        </is>
-      </c>
+      <c r="BI44" s="214" t="n"/>
       <c r="BJ44" s="145" t="n"/>
-      <c r="BK44" s="178" t="inlineStr">
-        <is>
-          <t>OBSERVACIONES</t>
-        </is>
-      </c>
+      <c r="BK44" s="178" t="n"/>
       <c r="BL44" s="64" t="n"/>
     </row>
     <row r="45" ht="42.6" customHeight="1" s="147">
@@ -27933,16 +27726,8 @@
       <c r="BF45" s="214" t="n"/>
       <c r="BG45" s="214" t="n"/>
       <c r="BH45" s="220" t="n"/>
-      <c r="BI45" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL AUSENCIAS</t>
-        </is>
-      </c>
-      <c r="BJ45" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL TARDANZAS</t>
-        </is>
-      </c>
+      <c r="BI45" s="2" t="n"/>
+      <c r="BJ45" s="2" t="n"/>
       <c r="BK45" s="154" t="n"/>
       <c r="BL45" s="64" t="n"/>
     </row>
@@ -28021,9 +27806,7 @@
         <v/>
       </c>
       <c r="BK46" s="220" t="n"/>
-      <c r="BL46" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="BL46" s="3" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1" s="147">
       <c r="A47" s="1" t="n">
@@ -28100,9 +27883,7 @@
         <v/>
       </c>
       <c r="BK47" s="220" t="n"/>
-      <c r="BL47" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="BL47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
@@ -28179,9 +27960,7 @@
         <v/>
       </c>
       <c r="BK48" s="220" t="n"/>
-      <c r="BL48" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="BL48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
@@ -28258,9 +28037,7 @@
         <v/>
       </c>
       <c r="BK49" s="220" t="n"/>
-      <c r="BL49" s="3" t="n">
-        <v>4</v>
-      </c>
+      <c r="BL49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
@@ -28337,9 +28114,7 @@
         <v/>
       </c>
       <c r="BK50" s="220" t="n"/>
-      <c r="BL50" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="BL50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
@@ -28416,9 +28191,7 @@
         <v/>
       </c>
       <c r="BK51" s="220" t="n"/>
-      <c r="BL51" s="3" t="n">
-        <v>6</v>
-      </c>
+      <c r="BL51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
@@ -28495,9 +28268,7 @@
         <v/>
       </c>
       <c r="BK52" s="220" t="n"/>
-      <c r="BL52" s="3" t="n">
-        <v>7</v>
-      </c>
+      <c r="BL52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
@@ -28574,9 +28345,7 @@
         <v/>
       </c>
       <c r="BK53" s="220" t="n"/>
-      <c r="BL53" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="BL53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
@@ -28653,9 +28422,7 @@
         <v/>
       </c>
       <c r="BK54" s="220" t="n"/>
-      <c r="BL54" s="3" t="n">
-        <v>9</v>
-      </c>
+      <c r="BL54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
@@ -34723,7 +34490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EE48"/>
+  <dimension ref="A1:EE54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="2.77734375" bestFit="1" customWidth="1" style="147" min="1" max="1"/>
@@ -37080,12 +36847,8 @@
         <v/>
       </c>
       <c r="AF15" s="220" t="n"/>
-      <c r="AG15" s="220" t="n">
-        <v>11</v>
-      </c>
-      <c r="AH15" s="220" t="n">
-        <v>11</v>
-      </c>
+      <c r="AG15" s="220" t="n"/>
+      <c r="AH15" s="220" t="n"/>
       <c r="AI15" s="220">
         <f>IF('MAESTRO 1°'!B15="","",'MAESTRO 1°'!B15)</f>
         <v/>
@@ -37124,12 +36887,8 @@
         <v/>
       </c>
       <c r="BN15" s="220" t="n"/>
-      <c r="BO15" s="220" t="n">
-        <v>11</v>
-      </c>
-      <c r="BP15" s="220" t="n">
-        <v>11</v>
-      </c>
+      <c r="BO15" s="220" t="n"/>
+      <c r="BP15" s="220" t="n"/>
       <c r="BQ15" s="220">
         <f>IF('MAESTRO 1°'!B15="","",'MAESTRO 1°'!B15)</f>
         <v/>
@@ -37229,12 +36988,8 @@
         <v/>
       </c>
       <c r="AF16" s="220" t="n"/>
-      <c r="AG16" s="220" t="n">
-        <v>12</v>
-      </c>
-      <c r="AH16" s="220" t="n">
-        <v>12</v>
-      </c>
+      <c r="AG16" s="220" t="n"/>
+      <c r="AH16" s="220" t="n"/>
       <c r="AI16" s="220">
         <f>IF('MAESTRO 1°'!B16="","",'MAESTRO 1°'!B16)</f>
         <v/>
@@ -37273,12 +37028,8 @@
         <v/>
       </c>
       <c r="BN16" s="220" t="n"/>
-      <c r="BO16" s="220" t="n">
-        <v>12</v>
-      </c>
-      <c r="BP16" s="220" t="n">
-        <v>12</v>
-      </c>
+      <c r="BO16" s="220" t="n"/>
+      <c r="BP16" s="220" t="n"/>
       <c r="BQ16" s="220">
         <f>IF('MAESTRO 1°'!B16="","",'MAESTRO 1°'!B16)</f>
         <v/>
@@ -37378,12 +37129,8 @@
         <v/>
       </c>
       <c r="AF17" s="220" t="n"/>
-      <c r="AG17" s="220" t="n">
-        <v>13</v>
-      </c>
-      <c r="AH17" s="220" t="n">
-        <v>13</v>
-      </c>
+      <c r="AG17" s="220" t="n"/>
+      <c r="AH17" s="220" t="n"/>
       <c r="AI17" s="220">
         <f>IF('MAESTRO 1°'!B17="","",'MAESTRO 1°'!B17)</f>
         <v/>
@@ -37422,12 +37169,8 @@
         <v/>
       </c>
       <c r="BN17" s="220" t="n"/>
-      <c r="BO17" s="220" t="n">
-        <v>13</v>
-      </c>
-      <c r="BP17" s="220" t="n">
-        <v>13</v>
-      </c>
+      <c r="BO17" s="220" t="n"/>
+      <c r="BP17" s="220" t="n"/>
       <c r="BQ17" s="220">
         <f>IF('MAESTRO 1°'!B17="","",'MAESTRO 1°'!B17)</f>
         <v/>
@@ -37527,12 +37270,8 @@
         <v/>
       </c>
       <c r="AF18" s="220" t="n"/>
-      <c r="AG18" s="220" t="n">
-        <v>14</v>
-      </c>
-      <c r="AH18" s="220" t="n">
-        <v>14</v>
-      </c>
+      <c r="AG18" s="220" t="n"/>
+      <c r="AH18" s="220" t="n"/>
       <c r="AI18" s="220">
         <f>IF('MAESTRO 1°'!B18="","",'MAESTRO 1°'!B18)</f>
         <v/>
@@ -37571,12 +37310,8 @@
         <v/>
       </c>
       <c r="BN18" s="220" t="n"/>
-      <c r="BO18" s="220" t="n">
-        <v>14</v>
-      </c>
-      <c r="BP18" s="220" t="n">
-        <v>14</v>
-      </c>
+      <c r="BO18" s="220" t="n"/>
+      <c r="BP18" s="220" t="n"/>
       <c r="BQ18" s="220">
         <f>IF('MAESTRO 1°'!B18="","",'MAESTRO 1°'!B18)</f>
         <v/>
@@ -37676,12 +37411,8 @@
         <v/>
       </c>
       <c r="AF19" s="220" t="n"/>
-      <c r="AG19" s="220" t="n">
-        <v>15</v>
-      </c>
-      <c r="AH19" s="220" t="n">
-        <v>15</v>
-      </c>
+      <c r="AG19" s="220" t="n"/>
+      <c r="AH19" s="220" t="n"/>
       <c r="AI19" s="220">
         <f>IF('MAESTRO 1°'!B19="","",'MAESTRO 1°'!B19)</f>
         <v/>
@@ -37720,12 +37451,8 @@
         <v/>
       </c>
       <c r="BN19" s="220" t="n"/>
-      <c r="BO19" s="220" t="n">
-        <v>15</v>
-      </c>
-      <c r="BP19" s="220" t="n">
-        <v>15</v>
-      </c>
+      <c r="BO19" s="220" t="n"/>
+      <c r="BP19" s="220" t="n"/>
       <c r="BQ19" s="220">
         <f>IF('MAESTRO 1°'!B19="","",'MAESTRO 1°'!B19)</f>
         <v/>
@@ -37825,12 +37552,8 @@
         <v/>
       </c>
       <c r="AF20" s="220" t="n"/>
-      <c r="AG20" s="220" t="n">
-        <v>16</v>
-      </c>
-      <c r="AH20" s="220" t="n">
-        <v>16</v>
-      </c>
+      <c r="AG20" s="220" t="n"/>
+      <c r="AH20" s="220" t="n"/>
       <c r="AI20" s="220">
         <f>IF('MAESTRO 1°'!B20="","",'MAESTRO 1°'!B20)</f>
         <v/>
@@ -37869,12 +37592,8 @@
         <v/>
       </c>
       <c r="BN20" s="220" t="n"/>
-      <c r="BO20" s="220" t="n">
-        <v>16</v>
-      </c>
-      <c r="BP20" s="220" t="n">
-        <v>16</v>
-      </c>
+      <c r="BO20" s="220" t="n"/>
+      <c r="BP20" s="220" t="n"/>
       <c r="BQ20" s="220">
         <f>IF('MAESTRO 1°'!B20="","",'MAESTRO 1°'!B20)</f>
         <v/>
@@ -37974,12 +37693,8 @@
         <v/>
       </c>
       <c r="AF21" s="220" t="n"/>
-      <c r="AG21" s="220" t="n">
-        <v>17</v>
-      </c>
-      <c r="AH21" s="220" t="n">
-        <v>17</v>
-      </c>
+      <c r="AG21" s="220" t="n"/>
+      <c r="AH21" s="220" t="n"/>
       <c r="AI21" s="220">
         <f>IF('MAESTRO 1°'!B21="","",'MAESTRO 1°'!B21)</f>
         <v/>
@@ -38018,12 +37733,8 @@
         <v/>
       </c>
       <c r="BN21" s="220" t="n"/>
-      <c r="BO21" s="220" t="n">
-        <v>17</v>
-      </c>
-      <c r="BP21" s="220" t="n">
-        <v>17</v>
-      </c>
+      <c r="BO21" s="220" t="n"/>
+      <c r="BP21" s="220" t="n"/>
       <c r="BQ21" s="220">
         <f>IF('MAESTRO 1°'!B21="","",'MAESTRO 1°'!B21)</f>
         <v/>
@@ -38123,12 +37834,8 @@
         <v/>
       </c>
       <c r="AF22" s="220" t="n"/>
-      <c r="AG22" s="220" t="n">
-        <v>18</v>
-      </c>
-      <c r="AH22" s="220" t="n">
-        <v>18</v>
-      </c>
+      <c r="AG22" s="220" t="n"/>
+      <c r="AH22" s="220" t="n"/>
       <c r="AI22" s="220">
         <f>IF('MAESTRO 1°'!B22="","",'MAESTRO 1°'!B22)</f>
         <v/>
@@ -38167,12 +37874,8 @@
         <v/>
       </c>
       <c r="BN22" s="220" t="n"/>
-      <c r="BO22" s="220" t="n">
-        <v>18</v>
-      </c>
-      <c r="BP22" s="220" t="n">
-        <v>18</v>
-      </c>
+      <c r="BO22" s="220" t="n"/>
+      <c r="BP22" s="220" t="n"/>
       <c r="BQ22" s="220">
         <f>IF('MAESTRO 1°'!B22="","",'MAESTRO 1°'!B22)</f>
         <v/>
@@ -38272,12 +37975,8 @@
         <v/>
       </c>
       <c r="AF23" s="220" t="n"/>
-      <c r="AG23" s="220" t="n">
-        <v>19</v>
-      </c>
-      <c r="AH23" s="220" t="n">
-        <v>19</v>
-      </c>
+      <c r="AG23" s="220" t="n"/>
+      <c r="AH23" s="220" t="n"/>
       <c r="AI23" s="220">
         <f>IF('MAESTRO 1°'!B23="","",'MAESTRO 1°'!B23)</f>
         <v/>
@@ -38316,12 +38015,8 @@
         <v/>
       </c>
       <c r="BN23" s="220" t="n"/>
-      <c r="BO23" s="220" t="n">
-        <v>19</v>
-      </c>
-      <c r="BP23" s="220" t="n">
-        <v>19</v>
-      </c>
+      <c r="BO23" s="220" t="n"/>
+      <c r="BP23" s="220" t="n"/>
       <c r="BQ23" s="220">
         <f>IF('MAESTRO 1°'!B23="","",'MAESTRO 1°'!B23)</f>
         <v/>
@@ -38421,12 +38116,8 @@
         <v/>
       </c>
       <c r="AF24" s="220" t="n"/>
-      <c r="AG24" s="220" t="n">
-        <v>20</v>
-      </c>
-      <c r="AH24" s="220" t="n">
-        <v>20</v>
-      </c>
+      <c r="AG24" s="220" t="n"/>
+      <c r="AH24" s="220" t="n"/>
       <c r="AI24" s="220">
         <f>IF('MAESTRO 1°'!B24="","",'MAESTRO 1°'!B24)</f>
         <v/>
@@ -38465,12 +38156,8 @@
         <v/>
       </c>
       <c r="BN24" s="220" t="n"/>
-      <c r="BO24" s="220" t="n">
-        <v>20</v>
-      </c>
-      <c r="BP24" s="220" t="n">
-        <v>20</v>
-      </c>
+      <c r="BO24" s="220" t="n"/>
+      <c r="BP24" s="220" t="n"/>
       <c r="BQ24" s="220">
         <f>IF('MAESTRO 1°'!B24="","",'MAESTRO 1°'!B24)</f>
         <v/>
@@ -38570,12 +38257,8 @@
         <v/>
       </c>
       <c r="AF25" s="220" t="n"/>
-      <c r="AG25" s="220" t="n">
-        <v>21</v>
-      </c>
-      <c r="AH25" s="220" t="n">
-        <v>21</v>
-      </c>
+      <c r="AG25" s="220" t="n"/>
+      <c r="AH25" s="220" t="n"/>
       <c r="AI25" s="220">
         <f>IF('MAESTRO 1°'!B25="","",'MAESTRO 1°'!B25)</f>
         <v/>
@@ -38614,12 +38297,8 @@
         <v/>
       </c>
       <c r="BN25" s="220" t="n"/>
-      <c r="BO25" s="220" t="n">
-        <v>21</v>
-      </c>
-      <c r="BP25" s="220" t="n">
-        <v>21</v>
-      </c>
+      <c r="BO25" s="220" t="n"/>
+      <c r="BP25" s="220" t="n"/>
       <c r="BQ25" s="220">
         <f>IF('MAESTRO 1°'!B25="","",'MAESTRO 1°'!B25)</f>
         <v/>
@@ -38719,12 +38398,8 @@
         <v/>
       </c>
       <c r="AF26" s="220" t="n"/>
-      <c r="AG26" s="220" t="n">
-        <v>22</v>
-      </c>
-      <c r="AH26" s="220" t="n">
-        <v>22</v>
-      </c>
+      <c r="AG26" s="220" t="n"/>
+      <c r="AH26" s="220" t="n"/>
       <c r="AI26" s="220">
         <f>IF('MAESTRO 1°'!B26="","",'MAESTRO 1°'!B26)</f>
         <v/>
@@ -38763,12 +38438,8 @@
         <v/>
       </c>
       <c r="BN26" s="220" t="n"/>
-      <c r="BO26" s="220" t="n">
-        <v>22</v>
-      </c>
-      <c r="BP26" s="220" t="n">
-        <v>22</v>
-      </c>
+      <c r="BO26" s="220" t="n"/>
+      <c r="BP26" s="220" t="n"/>
       <c r="BQ26" s="220">
         <f>IF('MAESTRO 1°'!B26="","",'MAESTRO 1°'!B26)</f>
         <v/>
@@ -38868,12 +38539,8 @@
         <v/>
       </c>
       <c r="AF27" s="220" t="n"/>
-      <c r="AG27" s="220" t="n">
-        <v>23</v>
-      </c>
-      <c r="AH27" s="220" t="n">
-        <v>23</v>
-      </c>
+      <c r="AG27" s="220" t="n"/>
+      <c r="AH27" s="220" t="n"/>
       <c r="AI27" s="220">
         <f>IF('MAESTRO 1°'!B27="","",'MAESTRO 1°'!B27)</f>
         <v/>
@@ -38912,12 +38579,8 @@
         <v/>
       </c>
       <c r="BN27" s="220" t="n"/>
-      <c r="BO27" s="220" t="n">
-        <v>23</v>
-      </c>
-      <c r="BP27" s="220" t="n">
-        <v>23</v>
-      </c>
+      <c r="BO27" s="220" t="n"/>
+      <c r="BP27" s="220" t="n"/>
       <c r="BQ27" s="220">
         <f>IF('MAESTRO 1°'!B27="","",'MAESTRO 1°'!B27)</f>
         <v/>
@@ -39017,12 +38680,8 @@
         <v/>
       </c>
       <c r="AF28" s="220" t="n"/>
-      <c r="AG28" s="220" t="n">
-        <v>24</v>
-      </c>
-      <c r="AH28" s="220" t="n">
-        <v>24</v>
-      </c>
+      <c r="AG28" s="220" t="n"/>
+      <c r="AH28" s="220" t="n"/>
       <c r="AI28" s="220">
         <f>IF('MAESTRO 1°'!B28="","",'MAESTRO 1°'!B28)</f>
         <v/>
@@ -39061,12 +38720,8 @@
         <v/>
       </c>
       <c r="BN28" s="220" t="n"/>
-      <c r="BO28" s="220" t="n">
-        <v>24</v>
-      </c>
-      <c r="BP28" s="220" t="n">
-        <v>24</v>
-      </c>
+      <c r="BO28" s="220" t="n"/>
+      <c r="BP28" s="220" t="n"/>
       <c r="BQ28" s="220">
         <f>IF('MAESTRO 1°'!B28="","",'MAESTRO 1°'!B28)</f>
         <v/>
@@ -39166,12 +38821,8 @@
         <v/>
       </c>
       <c r="AF29" s="220" t="n"/>
-      <c r="AG29" s="220" t="n">
-        <v>25</v>
-      </c>
-      <c r="AH29" s="220" t="n">
-        <v>25</v>
-      </c>
+      <c r="AG29" s="220" t="n"/>
+      <c r="AH29" s="220" t="n"/>
       <c r="AI29" s="220">
         <f>IF('MAESTRO 1°'!B29="","",'MAESTRO 1°'!B29)</f>
         <v/>
@@ -39210,12 +38861,8 @@
         <v/>
       </c>
       <c r="BN29" s="220" t="n"/>
-      <c r="BO29" s="220" t="n">
-        <v>25</v>
-      </c>
-      <c r="BP29" s="220" t="n">
-        <v>25</v>
-      </c>
+      <c r="BO29" s="220" t="n"/>
+      <c r="BP29" s="220" t="n"/>
       <c r="BQ29" s="220">
         <f>IF('MAESTRO 1°'!B29="","",'MAESTRO 1°'!B29)</f>
         <v/>
@@ -39315,12 +38962,8 @@
         <v/>
       </c>
       <c r="AF30" s="220" t="n"/>
-      <c r="AG30" s="220" t="n">
-        <v>26</v>
-      </c>
-      <c r="AH30" s="220" t="n">
-        <v>26</v>
-      </c>
+      <c r="AG30" s="220" t="n"/>
+      <c r="AH30" s="220" t="n"/>
       <c r="AI30" s="220">
         <f>IF('MAESTRO 1°'!B30="","",'MAESTRO 1°'!B30)</f>
         <v/>
@@ -39359,12 +39002,8 @@
         <v/>
       </c>
       <c r="BN30" s="220" t="n"/>
-      <c r="BO30" s="220" t="n">
-        <v>26</v>
-      </c>
-      <c r="BP30" s="220" t="n">
-        <v>26</v>
-      </c>
+      <c r="BO30" s="220" t="n"/>
+      <c r="BP30" s="220" t="n"/>
       <c r="BQ30" s="220">
         <f>IF('MAESTRO 1°'!B30="","",'MAESTRO 1°'!B30)</f>
         <v/>
@@ -39464,12 +39103,8 @@
         <v/>
       </c>
       <c r="AF31" s="220" t="n"/>
-      <c r="AG31" s="220" t="n">
-        <v>27</v>
-      </c>
-      <c r="AH31" s="220" t="n">
-        <v>27</v>
-      </c>
+      <c r="AG31" s="220" t="n"/>
+      <c r="AH31" s="220" t="n"/>
       <c r="AI31" s="220">
         <f>IF('MAESTRO 1°'!B31="","",'MAESTRO 1°'!B31)</f>
         <v/>
@@ -39508,12 +39143,8 @@
         <v/>
       </c>
       <c r="BN31" s="220" t="n"/>
-      <c r="BO31" s="220" t="n">
-        <v>27</v>
-      </c>
-      <c r="BP31" s="220" t="n">
-        <v>27</v>
-      </c>
+      <c r="BO31" s="220" t="n"/>
+      <c r="BP31" s="220" t="n"/>
       <c r="BQ31" s="220">
         <f>IF('MAESTRO 1°'!B31="","",'MAESTRO 1°'!B31)</f>
         <v/>
@@ -39613,12 +39244,8 @@
         <v/>
       </c>
       <c r="AF32" s="220" t="n"/>
-      <c r="AG32" s="220" t="n">
-        <v>28</v>
-      </c>
-      <c r="AH32" s="220" t="n">
-        <v>28</v>
-      </c>
+      <c r="AG32" s="220" t="n"/>
+      <c r="AH32" s="220" t="n"/>
       <c r="AI32" s="220">
         <f>IF('MAESTRO 1°'!B32="","",'MAESTRO 1°'!B32)</f>
         <v/>
@@ -39657,12 +39284,8 @@
         <v/>
       </c>
       <c r="BN32" s="220" t="n"/>
-      <c r="BO32" s="220" t="n">
-        <v>28</v>
-      </c>
-      <c r="BP32" s="220" t="n">
-        <v>28</v>
-      </c>
+      <c r="BO32" s="220" t="n"/>
+      <c r="BP32" s="220" t="n"/>
       <c r="BQ32" s="220">
         <f>IF('MAESTRO 1°'!B32="","",'MAESTRO 1°'!B32)</f>
         <v/>
@@ -39762,12 +39385,8 @@
         <v/>
       </c>
       <c r="AF33" s="220" t="n"/>
-      <c r="AG33" s="220" t="n">
-        <v>29</v>
-      </c>
-      <c r="AH33" s="220" t="n">
-        <v>29</v>
-      </c>
+      <c r="AG33" s="220" t="n"/>
+      <c r="AH33" s="220" t="n"/>
       <c r="AI33" s="220">
         <f>IF('MAESTRO 1°'!B33="","",'MAESTRO 1°'!B33)</f>
         <v/>
@@ -39806,12 +39425,8 @@
         <v/>
       </c>
       <c r="BN33" s="220" t="n"/>
-      <c r="BO33" s="220" t="n">
-        <v>29</v>
-      </c>
-      <c r="BP33" s="220" t="n">
-        <v>29</v>
-      </c>
+      <c r="BO33" s="220" t="n"/>
+      <c r="BP33" s="220" t="n"/>
       <c r="BQ33" s="220">
         <f>IF('MAESTRO 1°'!B33="","",'MAESTRO 1°'!B33)</f>
         <v/>
@@ -39911,12 +39526,8 @@
         <v/>
       </c>
       <c r="AF34" s="220" t="n"/>
-      <c r="AG34" s="220" t="n">
-        <v>30</v>
-      </c>
-      <c r="AH34" s="220" t="n">
-        <v>30</v>
-      </c>
+      <c r="AG34" s="220" t="n"/>
+      <c r="AH34" s="220" t="n"/>
       <c r="AI34" s="220">
         <f>IF('MAESTRO 1°'!B34="","",'MAESTRO 1°'!B34)</f>
         <v/>
@@ -39955,12 +39566,8 @@
         <v/>
       </c>
       <c r="BN34" s="220" t="n"/>
-      <c r="BO34" s="220" t="n">
-        <v>30</v>
-      </c>
-      <c r="BP34" s="220" t="n">
-        <v>30</v>
-      </c>
+      <c r="BO34" s="220" t="n"/>
+      <c r="BP34" s="220" t="n"/>
       <c r="BQ34" s="220">
         <f>IF('MAESTRO 1°'!B34="","",'MAESTRO 1°'!B34)</f>
         <v/>
@@ -40060,12 +39667,8 @@
         <v/>
       </c>
       <c r="AF35" s="220" t="n"/>
-      <c r="AG35" s="220" t="n">
-        <v>31</v>
-      </c>
-      <c r="AH35" s="220" t="n">
-        <v>31</v>
-      </c>
+      <c r="AG35" s="220" t="n"/>
+      <c r="AH35" s="220" t="n"/>
       <c r="AI35" s="220">
         <f>IF('MAESTRO 1°'!B35="","",'MAESTRO 1°'!B35)</f>
         <v/>
@@ -40104,12 +39707,8 @@
         <v/>
       </c>
       <c r="BN35" s="220" t="n"/>
-      <c r="BO35" s="220" t="n">
-        <v>31</v>
-      </c>
-      <c r="BP35" s="220" t="n">
-        <v>31</v>
-      </c>
+      <c r="BO35" s="220" t="n"/>
+      <c r="BP35" s="220" t="n"/>
       <c r="BQ35" s="220">
         <f>IF('MAESTRO 1°'!B35="","",'MAESTRO 1°'!B35)</f>
         <v/>
@@ -40209,12 +39808,8 @@
         <v/>
       </c>
       <c r="AF36" s="220" t="n"/>
-      <c r="AG36" s="220" t="n">
-        <v>32</v>
-      </c>
-      <c r="AH36" s="220" t="n">
-        <v>32</v>
-      </c>
+      <c r="AG36" s="220" t="n"/>
+      <c r="AH36" s="220" t="n"/>
       <c r="AI36" s="220">
         <f>IF('MAESTRO 1°'!B36="","",'MAESTRO 1°'!B36)</f>
         <v/>
@@ -40253,12 +39848,8 @@
         <v/>
       </c>
       <c r="BN36" s="220" t="n"/>
-      <c r="BO36" s="220" t="n">
-        <v>32</v>
-      </c>
-      <c r="BP36" s="220" t="n">
-        <v>32</v>
-      </c>
+      <c r="BO36" s="220" t="n"/>
+      <c r="BP36" s="220" t="n"/>
       <c r="BQ36" s="220">
         <f>IF('MAESTRO 1°'!B36="","",'MAESTRO 1°'!B36)</f>
         <v/>
@@ -40358,12 +39949,8 @@
         <v/>
       </c>
       <c r="AF37" s="220" t="n"/>
-      <c r="AG37" s="220" t="n">
-        <v>33</v>
-      </c>
-      <c r="AH37" s="220" t="n">
-        <v>33</v>
-      </c>
+      <c r="AG37" s="220" t="n"/>
+      <c r="AH37" s="220" t="n"/>
       <c r="AI37" s="220">
         <f>IF('MAESTRO 1°'!B37="","",'MAESTRO 1°'!B37)</f>
         <v/>
@@ -40402,12 +39989,8 @@
         <v/>
       </c>
       <c r="BN37" s="220" t="n"/>
-      <c r="BO37" s="220" t="n">
-        <v>33</v>
-      </c>
-      <c r="BP37" s="220" t="n">
-        <v>33</v>
-      </c>
+      <c r="BO37" s="220" t="n"/>
+      <c r="BP37" s="220" t="n"/>
       <c r="BQ37" s="220">
         <f>IF('MAESTRO 1°'!B37="","",'MAESTRO 1°'!B37)</f>
         <v/>
@@ -40507,12 +40090,8 @@
         <v/>
       </c>
       <c r="AF38" s="220" t="n"/>
-      <c r="AG38" s="220" t="n">
-        <v>34</v>
-      </c>
-      <c r="AH38" s="220" t="n">
-        <v>34</v>
-      </c>
+      <c r="AG38" s="220" t="n"/>
+      <c r="AH38" s="220" t="n"/>
       <c r="AI38" s="220">
         <f>IF('MAESTRO 1°'!B38="","",'MAESTRO 1°'!B38)</f>
         <v/>
@@ -40551,12 +40130,8 @@
         <v/>
       </c>
       <c r="BN38" s="220" t="n"/>
-      <c r="BO38" s="220" t="n">
-        <v>34</v>
-      </c>
-      <c r="BP38" s="220" t="n">
-        <v>34</v>
-      </c>
+      <c r="BO38" s="220" t="n"/>
+      <c r="BP38" s="220" t="n"/>
       <c r="BQ38" s="220">
         <f>IF('MAESTRO 1°'!B38="","",'MAESTRO 1°'!B38)</f>
         <v/>
@@ -40656,32 +40231,16 @@
         <v/>
       </c>
       <c r="AF39" s="220" t="n"/>
-      <c r="AG39" s="220" t="n">
-        <v>35</v>
-      </c>
-      <c r="AH39" s="220" t="n">
-        <v>35</v>
-      </c>
+      <c r="AG39" s="220" t="n"/>
+      <c r="AH39" s="220" t="n"/>
       <c r="AI39" s="220">
         <f>IF('MAESTRO 1°'!B39="","",'MAESTRO 1°'!B39)</f>
         <v/>
       </c>
       <c r="AJ39" s="145" t="n"/>
-      <c r="AK39" s="97" t="inlineStr">
-        <is>
-          <t>Actividad 37</t>
-        </is>
-      </c>
-      <c r="AL39" s="97" t="inlineStr">
-        <is>
-          <t>Actividad 38</t>
-        </is>
-      </c>
-      <c r="AM39" s="97" t="inlineStr">
-        <is>
-          <t>Actividad 39</t>
-        </is>
-      </c>
+      <c r="AK39" s="97" t="n"/>
+      <c r="AL39" s="97" t="n"/>
+      <c r="AM39" s="97" t="n"/>
       <c r="AN39" s="97" t="n"/>
       <c r="AO39" s="97" t="n"/>
       <c r="AP39" s="97" t="n"/>
@@ -40693,21 +40252,9 @@
       <c r="AV39" s="97" t="n"/>
       <c r="AW39" s="97" t="n"/>
       <c r="AX39" s="97" t="n"/>
-      <c r="AY39" s="97" t="inlineStr">
-        <is>
-          <t>Actividad 51</t>
-        </is>
-      </c>
-      <c r="AZ39" s="97" t="inlineStr">
-        <is>
-          <t>Actividad 52</t>
-        </is>
-      </c>
-      <c r="BA39" s="97" t="inlineStr">
-        <is>
-          <t>Actividad 53</t>
-        </is>
-      </c>
+      <c r="AY39" s="97" t="n"/>
+      <c r="AZ39" s="97" t="n"/>
+      <c r="BA39" s="97" t="n"/>
       <c r="BB39" s="97" t="n"/>
       <c r="BC39" s="97" t="n"/>
       <c r="BD39" s="97" t="n"/>
@@ -40724,12 +40271,8 @@
         <v/>
       </c>
       <c r="BN39" s="220" t="n"/>
-      <c r="BO39" s="220" t="n">
-        <v>35</v>
-      </c>
-      <c r="BP39" s="220" t="n">
-        <v>35</v>
-      </c>
+      <c r="BO39" s="220" t="n"/>
+      <c r="BP39" s="220" t="n"/>
       <c r="BQ39" s="220">
         <f>IF('MAESTRO 1°'!B39="","",'MAESTRO 1°'!B39)</f>
         <v/>
@@ -40827,11 +40370,7 @@
           <t>Actividad 4</t>
         </is>
       </c>
-      <c r="E40" s="264" t="inlineStr">
-        <is>
-          <t>Actividad 5</t>
-        </is>
-      </c>
+      <c r="E40" s="264" t="n"/>
       <c r="F40" s="227" t="n"/>
       <c r="G40" s="227" t="n"/>
       <c r="H40" s="227" t="n"/>
@@ -40844,21 +40383,9 @@
       <c r="O40" s="227" t="n"/>
       <c r="P40" s="227" t="n"/>
       <c r="Q40" s="227" t="n"/>
-      <c r="R40" s="227" t="inlineStr">
-        <is>
-          <t>Actividad 18</t>
-        </is>
-      </c>
-      <c r="S40" s="227" t="inlineStr">
-        <is>
-          <t>Actividad 19</t>
-        </is>
-      </c>
-      <c r="T40" s="227" t="inlineStr">
-        <is>
-          <t>Actividad 20</t>
-        </is>
-      </c>
+      <c r="R40" s="227" t="n"/>
+      <c r="S40" s="227" t="n"/>
+      <c r="T40" s="227" t="n"/>
       <c r="U40" s="227" t="n"/>
       <c r="V40" s="227" t="n"/>
       <c r="W40" s="227" t="n"/>
@@ -40871,12 +40398,8 @@
       <c r="AD40" s="227" t="n"/>
       <c r="AE40" s="42" t="n"/>
       <c r="AF40" s="220" t="n"/>
-      <c r="AG40" s="220" t="n">
-        <v>36</v>
-      </c>
-      <c r="AH40" s="220" t="n">
-        <v>36</v>
-      </c>
+      <c r="AG40" s="220" t="n"/>
+      <c r="AH40" s="220" t="n"/>
       <c r="AI40" s="220" t="n"/>
       <c r="AJ40" s="145" t="n"/>
       <c r="AK40" s="221" t="n"/>
@@ -40909,12 +40432,8 @@
       <c r="BL40" s="221" t="n"/>
       <c r="BM40" s="20" t="n"/>
       <c r="BN40" s="220" t="n"/>
-      <c r="BO40" s="220" t="n">
-        <v>36</v>
-      </c>
-      <c r="BP40" s="220" t="n">
-        <v>36</v>
-      </c>
+      <c r="BO40" s="220" t="n"/>
+      <c r="BP40" s="220" t="n"/>
       <c r="BQ40" s="220">
         <f>IF('MAESTRO 1°'!B40="","",'MAESTRO 1°'!B40)</f>
         <v/>
@@ -41005,12 +40524,8 @@
       <c r="AD41" s="222" t="n"/>
       <c r="AE41" s="42" t="n"/>
       <c r="AF41" s="220" t="n"/>
-      <c r="AG41" s="220" t="n">
-        <v>37</v>
-      </c>
-      <c r="AH41" s="220" t="n">
-        <v>37</v>
-      </c>
+      <c r="AG41" s="220" t="n"/>
+      <c r="AH41" s="220" t="n"/>
       <c r="AI41" s="220" t="n"/>
       <c r="AJ41" s="145" t="n"/>
       <c r="AK41" s="222" t="n"/>
@@ -41043,12 +40558,8 @@
       <c r="BL41" s="222" t="n"/>
       <c r="BM41" s="20" t="n"/>
       <c r="BN41" s="220" t="n"/>
-      <c r="BO41" s="220" t="n">
-        <v>37</v>
-      </c>
-      <c r="BP41" s="220" t="n">
-        <v>37</v>
-      </c>
+      <c r="BO41" s="220" t="n"/>
+      <c r="BP41" s="220" t="n"/>
       <c r="BQ41" s="220">
         <f>IF('MAESTRO 1°'!B41="","",'MAESTRO 1°'!B41)</f>
         <v/>
@@ -41139,12 +40650,8 @@
       <c r="AD42" s="222" t="n"/>
       <c r="AE42" s="42" t="n"/>
       <c r="AF42" s="220" t="n"/>
-      <c r="AG42" s="220" t="n">
-        <v>38</v>
-      </c>
-      <c r="AH42" s="220" t="n">
-        <v>38</v>
-      </c>
+      <c r="AG42" s="220" t="n"/>
+      <c r="AH42" s="220" t="n"/>
       <c r="AI42" s="220" t="n"/>
       <c r="AJ42" s="145" t="n"/>
       <c r="AK42" s="222" t="n"/>
@@ -41177,12 +40684,8 @@
       <c r="BL42" s="222" t="n"/>
       <c r="BM42" s="20" t="n"/>
       <c r="BN42" s="220" t="n"/>
-      <c r="BO42" s="220" t="n">
-        <v>38</v>
-      </c>
-      <c r="BP42" s="220" t="n">
-        <v>38</v>
-      </c>
+      <c r="BO42" s="220" t="n"/>
+      <c r="BP42" s="220" t="n"/>
       <c r="BQ42" s="220">
         <f>IF('MAESTRO 1°'!B42="","",'MAESTRO 1°'!B42)</f>
         <v/>
@@ -41273,12 +40776,8 @@
       <c r="AD43" s="222" t="n"/>
       <c r="AE43" s="42" t="n"/>
       <c r="AF43" s="220" t="n"/>
-      <c r="AG43" s="220" t="n">
-        <v>39</v>
-      </c>
-      <c r="AH43" s="220" t="n">
-        <v>39</v>
-      </c>
+      <c r="AG43" s="220" t="n"/>
+      <c r="AH43" s="220" t="n"/>
       <c r="AI43" s="220" t="n"/>
       <c r="AJ43" s="145" t="n"/>
       <c r="AK43" s="222" t="n"/>
@@ -41311,12 +40810,8 @@
       <c r="BL43" s="222" t="n"/>
       <c r="BM43" s="20" t="n"/>
       <c r="BN43" s="220" t="n"/>
-      <c r="BO43" s="220" t="n">
-        <v>39</v>
-      </c>
-      <c r="BP43" s="220" t="n">
-        <v>39</v>
-      </c>
+      <c r="BO43" s="220" t="n"/>
+      <c r="BP43" s="220" t="n"/>
       <c r="BQ43" s="220">
         <f>IF('MAESTRO 1°'!B43="","",'MAESTRO 1°'!B43)</f>
         <v/>
@@ -41407,12 +40902,8 @@
       <c r="AD44" s="222" t="n"/>
       <c r="AE44" s="20" t="n"/>
       <c r="AF44" s="220" t="n"/>
-      <c r="AG44" s="220" t="n">
-        <v>40</v>
-      </c>
-      <c r="AH44" s="220" t="n">
-        <v>40</v>
-      </c>
+      <c r="AG44" s="220" t="n"/>
+      <c r="AH44" s="220" t="n"/>
       <c r="AI44" s="220" t="n"/>
       <c r="AJ44" s="145" t="n"/>
       <c r="AK44" s="222" t="n"/>
@@ -41445,12 +40936,8 @@
       <c r="BL44" s="222" t="n"/>
       <c r="BM44" s="20" t="n"/>
       <c r="BN44" s="220" t="n"/>
-      <c r="BO44" s="220" t="n">
-        <v>40</v>
-      </c>
-      <c r="BP44" s="220" t="n">
-        <v>40</v>
-      </c>
+      <c r="BO44" s="220" t="n"/>
+      <c r="BP44" s="220" t="n"/>
       <c r="BQ44" s="220">
         <f>IF('MAESTRO 1°'!B44="","",'MAESTRO 1°'!B44)</f>
         <v/>
@@ -41541,12 +41028,8 @@
       <c r="AD45" s="222" t="n"/>
       <c r="AE45" s="20" t="n"/>
       <c r="AF45" s="220" t="n"/>
-      <c r="AG45" s="220" t="n">
-        <v>41</v>
-      </c>
-      <c r="AH45" s="220" t="n">
-        <v>41</v>
-      </c>
+      <c r="AG45" s="220" t="n"/>
+      <c r="AH45" s="220" t="n"/>
       <c r="AI45" s="220" t="n"/>
       <c r="AJ45" s="145" t="n"/>
       <c r="AK45" s="222" t="n"/>
@@ -41579,12 +41062,8 @@
       <c r="BL45" s="222" t="n"/>
       <c r="BM45" s="20" t="n"/>
       <c r="BN45" s="220" t="n"/>
-      <c r="BO45" s="220" t="n">
-        <v>41</v>
-      </c>
-      <c r="BP45" s="220" t="n">
-        <v>41</v>
-      </c>
+      <c r="BO45" s="220" t="n"/>
+      <c r="BP45" s="220" t="n"/>
       <c r="BQ45" s="220" t="n"/>
       <c r="BR45" s="145" t="n"/>
       <c r="BS45" s="162" t="n"/>
@@ -41672,12 +41151,8 @@
       <c r="AD46" s="222" t="n"/>
       <c r="AE46" s="20" t="n"/>
       <c r="AF46" s="220" t="n"/>
-      <c r="AG46" s="220" t="n">
-        <v>42</v>
-      </c>
-      <c r="AH46" s="220" t="n">
-        <v>42</v>
-      </c>
+      <c r="AG46" s="220" t="n"/>
+      <c r="AH46" s="220" t="n"/>
       <c r="AI46" s="220" t="n"/>
       <c r="AJ46" s="145" t="n"/>
       <c r="AK46" s="222" t="n"/>
@@ -41710,12 +41185,8 @@
       <c r="BL46" s="222" t="n"/>
       <c r="BM46" s="20" t="n"/>
       <c r="BN46" s="220" t="n"/>
-      <c r="BO46" s="220" t="n">
-        <v>42</v>
-      </c>
-      <c r="BP46" s="220" t="n">
-        <v>42</v>
-      </c>
+      <c r="BO46" s="220" t="n"/>
+      <c r="BP46" s="220" t="n"/>
       <c r="BQ46" s="220" t="n"/>
       <c r="BR46" s="145" t="n"/>
       <c r="BS46" s="162" t="n"/>
@@ -41803,12 +41274,8 @@
       <c r="AD47" s="222" t="n"/>
       <c r="AE47" s="20" t="n"/>
       <c r="AF47" s="220" t="n"/>
-      <c r="AG47" s="220" t="n">
-        <v>43</v>
-      </c>
-      <c r="AH47" s="220" t="n">
-        <v>43</v>
-      </c>
+      <c r="AG47" s="220" t="n"/>
+      <c r="AH47" s="220" t="n"/>
       <c r="AI47" s="220" t="n"/>
       <c r="AJ47" s="145" t="n"/>
       <c r="AK47" s="222" t="n"/>
@@ -41841,12 +41308,8 @@
       <c r="BL47" s="222" t="n"/>
       <c r="BM47" s="20" t="n"/>
       <c r="BN47" s="220" t="n"/>
-      <c r="BO47" s="220" t="n">
-        <v>43</v>
-      </c>
-      <c r="BP47" s="220" t="n">
-        <v>43</v>
-      </c>
+      <c r="BO47" s="220" t="n"/>
+      <c r="BP47" s="220" t="n"/>
       <c r="BQ47" s="220" t="n"/>
       <c r="BR47" s="145" t="n"/>
       <c r="BS47" s="162" t="n"/>
@@ -41934,12 +41397,8 @@
       <c r="AD48" s="223" t="n"/>
       <c r="AE48" s="20" t="n"/>
       <c r="AF48" s="220" t="n"/>
-      <c r="AG48" s="220" t="n">
-        <v>44</v>
-      </c>
-      <c r="AH48" s="220" t="n">
-        <v>44</v>
-      </c>
+      <c r="AG48" s="220" t="n"/>
+      <c r="AH48" s="220" t="n"/>
       <c r="AI48" s="220" t="n"/>
       <c r="AJ48" s="145" t="n"/>
       <c r="AK48" s="223" t="n"/>
@@ -41972,12 +41431,8 @@
       <c r="BL48" s="223" t="n"/>
       <c r="BM48" s="20" t="n"/>
       <c r="BN48" s="220" t="n"/>
-      <c r="BO48" s="220" t="n">
-        <v>44</v>
-      </c>
-      <c r="BP48" s="7" t="n">
-        <v>44</v>
-      </c>
+      <c r="BO48" s="220" t="n"/>
+      <c r="BP48" s="7" t="n"/>
       <c r="BQ48" s="220" t="n"/>
       <c r="BR48" s="145" t="n"/>
       <c r="BS48" s="154" t="n"/>
@@ -42030,6 +41485,12 @@
       <c r="EB48" s="148" t="n"/>
       <c r="EC48" s="148" t="n"/>
     </row>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
   </sheetData>
   <mergeCells count="260">
     <mergeCell ref="CA40:CA48"/>

</xml_diff>